<commit_message>
changes based on first revision
</commit_message>
<xml_diff>
--- a/data/generalprevs_allmodels_30yART2019.xlsx
+++ b/data/generalprevs_allmodels_30yART2019.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\CapeTown\UCT\projects\STI_HIV_Congress\Copied_Linux_thembisa\Linux_Themibsa\Rcode\Data_final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\CapeTown\UCT\projects\FSW_modelling\Analyses\Rcode\Data_final_rev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E833874E-8FDC-4FFF-9446-697C433546BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78392086-20A7-434E-B064-E41DD62DA54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mod1a" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="mod3b" sheetId="9" r:id="rId6"/>
     <sheet name="information" sheetId="8" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -9047,322 +9047,322 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>1.2401310900000009E-2</v>
+        <v>1.2763513099999972E-2</v>
       </c>
       <c r="C5">
-        <v>9.5012382100000042E-2</v>
+        <v>9.5068399500000234E-2</v>
       </c>
       <c r="D5">
-        <v>0.16655436300000009</v>
+        <v>0.16689155299999955</v>
       </c>
       <c r="E5">
-        <v>0.18482808100000025</v>
+        <v>0.19003523700000008</v>
       </c>
       <c r="F5">
-        <v>0.17428979599999983</v>
+        <v>0.18363493200000006</v>
       </c>
       <c r="G5">
-        <v>0.15386556500000051</v>
+        <v>0.16392175599999995</v>
       </c>
       <c r="H5">
-        <v>0.12491466700000017</v>
+        <v>0.13408317999999994</v>
       </c>
       <c r="I5">
-        <v>8.9801913900000155E-2</v>
+        <v>9.71986132000002E-2</v>
       </c>
       <c r="J5">
-        <v>7.667348210000019E-2</v>
+        <v>7.7263101899999978E-2</v>
       </c>
       <c r="K5">
-        <v>0.25567510300000057</v>
+        <v>0.25442985999999984</v>
       </c>
       <c r="L5">
-        <v>0.2545971990000005</v>
+        <v>0.25108339199999929</v>
       </c>
       <c r="M5">
-        <v>0.19670918999999995</v>
+        <v>0.19570686600000062</v>
       </c>
       <c r="N5">
-        <v>0.16263516799999969</v>
+        <v>0.16261315900000059</v>
       </c>
       <c r="O5">
-        <v>0.13118702500000021</v>
+        <v>0.13016951499999962</v>
       </c>
       <c r="P5">
-        <v>9.5139510399999919E-2</v>
+        <v>9.3509828400000466E-2</v>
       </c>
       <c r="Q5">
-        <v>6.0631115199999926E-2</v>
+        <v>5.919931069999966E-2</v>
       </c>
       <c r="R5">
-        <v>1.0057931510000001E-2</v>
+        <v>1.029809996999999E-2</v>
       </c>
       <c r="S5">
-        <v>8.7460895400000169E-2</v>
+        <v>8.789080519999995E-2</v>
       </c>
       <c r="T5">
-        <v>0.17804066500000035</v>
+        <v>0.17905510799999963</v>
       </c>
       <c r="U5">
-        <v>0.20595754300000027</v>
+        <v>0.20931093400000023</v>
       </c>
       <c r="V5">
-        <v>0.19337676600000012</v>
+        <v>0.19961450099999972</v>
       </c>
       <c r="W5">
-        <v>0.16605137399999956</v>
+        <v>0.17312967600000009</v>
       </c>
       <c r="X5">
-        <v>0.13619368399999965</v>
+        <v>0.14263815000000024</v>
       </c>
       <c r="Y5">
-        <v>0.10268031179999976</v>
+        <v>0.1079113607000005</v>
       </c>
       <c r="Z5">
-        <v>6.8518652500000193E-2</v>
+        <v>7.2268079599999771E-2</v>
       </c>
       <c r="AA5">
-        <v>6.800686750000004E-2</v>
+        <v>6.8349489799999857E-2</v>
       </c>
       <c r="AB5">
-        <v>0.25498142200000024</v>
+        <v>0.25486564800000078</v>
       </c>
       <c r="AC5">
-        <v>0.30856035799999987</v>
+        <v>0.30769112399999943</v>
       </c>
       <c r="AD5">
-        <v>0.25163483499999989</v>
+        <v>0.25012311099999956</v>
       </c>
       <c r="AE5">
-        <v>0.20286323700000028</v>
+        <v>0.2031472389999992</v>
       </c>
       <c r="AF5">
-        <v>0.16622128599999988</v>
+        <v>0.1659930360000002</v>
       </c>
       <c r="AG5">
-        <v>0.1270263939999999</v>
+        <v>0.12567798600000035</v>
       </c>
       <c r="AH5">
-        <v>8.6661771200000098E-2</v>
+        <v>8.490504980000016E-2</v>
       </c>
       <c r="AI5">
-        <v>5.1452290200000118E-2</v>
+        <v>5.0061709400000071E-2</v>
       </c>
       <c r="AJ5">
-        <v>9.5418753700000063E-3</v>
+        <v>9.5869605000000139E-3</v>
       </c>
       <c r="AK5">
-        <v>7.3101243799999799E-2</v>
+        <v>7.3184270200000026E-2</v>
       </c>
       <c r="AL5">
-        <v>0.16950454199999979</v>
+        <v>0.17064950199999993</v>
       </c>
       <c r="AM5">
-        <v>0.21534484399999962</v>
+        <v>0.21837431200000035</v>
       </c>
       <c r="AN5">
-        <v>0.20734869299999945</v>
+        <v>0.21170841099999935</v>
       </c>
       <c r="AO5">
-        <v>0.1762521490000005</v>
+        <v>0.18080942599999941</v>
       </c>
       <c r="AP5">
-        <v>0.14353541899999964</v>
+        <v>0.14733568699999985</v>
       </c>
       <c r="AQ5">
-        <v>0.11143991299999971</v>
+        <v>0.11421405899999995</v>
       </c>
       <c r="AR5">
-        <v>7.8648328799999875E-2</v>
+        <v>8.0442292499999846E-2</v>
       </c>
       <c r="AS5">
-        <v>5.9526841499999941E-2</v>
+        <v>5.9391695800000192E-2</v>
       </c>
       <c r="AT5">
-        <v>0.23240690400000036</v>
+        <v>0.23157394999999978</v>
       </c>
       <c r="AU5">
-        <v>0.32705817699999934</v>
+        <v>0.32799341899999779</v>
       </c>
       <c r="AV5">
-        <v>0.30194172900000005</v>
+        <v>0.30168413199999877</v>
       </c>
       <c r="AW5">
-        <v>0.24197344700000001</v>
+        <v>0.24204340100000124</v>
       </c>
       <c r="AX5">
-        <v>0.19664662100000019</v>
+        <v>0.19700105400000067</v>
       </c>
       <c r="AY5">
-        <v>0.15500598800000001</v>
+        <v>0.15420228299999969</v>
       </c>
       <c r="AZ5">
-        <v>0.11174079879999968</v>
+        <v>0.10989805589999949</v>
       </c>
       <c r="BA5">
-        <v>7.1339120600000097E-2</v>
+        <v>6.9340880000000049E-2</v>
       </c>
       <c r="BB5">
-        <v>1.4215154999999946E-2</v>
+        <v>1.4136273699999983E-2</v>
       </c>
       <c r="BC5">
-        <v>5.699361499999988E-2</v>
+        <v>5.6557465100000134E-2</v>
       </c>
       <c r="BD5">
-        <v>0.14411815199999997</v>
+        <v>0.14448682800000001</v>
       </c>
       <c r="BE5">
-        <v>0.2154845130000006</v>
+        <v>0.21840398099999964</v>
       </c>
       <c r="BF5">
-        <v>0.22482456299999948</v>
+        <v>0.22880806799999959</v>
       </c>
       <c r="BG5">
-        <v>0.19923893400000037</v>
+        <v>0.20268347400000092</v>
       </c>
       <c r="BH5">
-        <v>0.16177253699999997</v>
+        <v>0.16403859400000018</v>
       </c>
       <c r="BI5">
-        <v>0.12795823499999986</v>
+        <v>0.12905061500000017</v>
       </c>
       <c r="BJ5">
-        <v>9.6157026700000134E-2</v>
+        <v>9.6326203000000013E-2</v>
       </c>
       <c r="BK5">
-        <v>5.5442636999999829E-2</v>
+        <v>5.5068746600000121E-2</v>
       </c>
       <c r="BL5">
-        <v>0.19818276500000029</v>
+        <v>0.19585997900000082</v>
       </c>
       <c r="BM5">
-        <v>0.31054712000000045</v>
+        <v>0.31053211799999975</v>
       </c>
       <c r="BN5">
-        <v>0.35255480200000028</v>
+        <v>0.35468666099999874</v>
       </c>
       <c r="BO5">
-        <v>0.30599842699999963</v>
+        <v>0.30659231699999911</v>
       </c>
       <c r="BP5">
-        <v>0.24527652099999964</v>
+        <v>0.24579705399999896</v>
       </c>
       <c r="BQ5">
-        <v>0.19589381500000008</v>
+        <v>0.1957896879999991</v>
       </c>
       <c r="BR5">
-        <v>0.14924513999999989</v>
+        <v>0.1477036540000001</v>
       </c>
       <c r="BS5">
-        <v>0.10360485469999985</v>
+        <v>0.10107941779999957</v>
       </c>
       <c r="BT5">
-        <v>2.5435999399999919E-2</v>
+        <v>2.5434143800000059E-2</v>
       </c>
       <c r="BU5">
-        <v>4.604791559999992E-2</v>
+        <v>4.5464305800000035E-2</v>
       </c>
       <c r="BV5">
-        <v>0.10732285260000016</v>
+        <v>0.10680256329999988</v>
       </c>
       <c r="BW5">
-        <v>0.18655536600000025</v>
+        <v>0.18845513099999997</v>
       </c>
       <c r="BX5">
-        <v>0.23724358000000006</v>
+        <v>0.24132843700000067</v>
       </c>
       <c r="BY5">
-        <v>0.23202842100000026</v>
+        <v>0.23617487300000053</v>
       </c>
       <c r="BZ5">
-        <v>0.20036936799999963</v>
+        <v>0.20317201199999985</v>
       </c>
       <c r="CA5">
-        <v>0.16032295399999949</v>
+        <v>0.16154063800000051</v>
       </c>
       <c r="CB5">
-        <v>0.12537474600000009</v>
+        <v>0.12534508900000021</v>
       </c>
       <c r="CC5">
-        <v>5.9375021500000041E-2</v>
+        <v>5.9334782999999981E-2</v>
       </c>
       <c r="CD5">
-        <v>0.15794602900000002</v>
+        <v>0.15514757300000032</v>
       </c>
       <c r="CE5">
-        <v>0.26263029299999957</v>
+        <v>0.2601044699999997</v>
       </c>
       <c r="CF5">
-        <v>0.34694979799999848</v>
+        <v>0.34776795200000049</v>
       </c>
       <c r="CG5">
-        <v>0.37706431300000098</v>
+        <v>0.37997574900000186</v>
       </c>
       <c r="CH5">
-        <v>0.32514240300000002</v>
+        <v>0.32625780199999893</v>
       </c>
       <c r="CI5">
-        <v>0.25991396700000108</v>
+        <v>0.26039426000000054</v>
       </c>
       <c r="CJ5">
-        <v>0.20515551599999993</v>
+        <v>0.20464527200000024</v>
       </c>
       <c r="CK5">
-        <v>0.15482436200000019</v>
+        <v>0.15268942800000024</v>
       </c>
       <c r="CL5">
-        <v>2.9227160299999867E-2</v>
+        <v>2.935974649999995E-2</v>
       </c>
       <c r="CM5">
-        <v>4.3260579099999912E-2</v>
+        <v>4.3064920300000094E-2</v>
       </c>
       <c r="CN5">
-        <v>7.5476225899999791E-2</v>
+        <v>7.4738277900000344E-2</v>
       </c>
       <c r="CO5">
-        <v>0.13722318399999969</v>
+        <v>0.13778497699999978</v>
       </c>
       <c r="CP5">
-        <v>0.20472149199999953</v>
+        <v>0.20761888299999948</v>
       </c>
       <c r="CQ5">
-        <v>0.24309150300000001</v>
+        <v>0.2473370079999995</v>
       </c>
       <c r="CR5">
-        <v>0.23191846100000058</v>
+        <v>0.23577634700000039</v>
       </c>
       <c r="CS5">
-        <v>0.19811651699999983</v>
+        <v>0.20040107299999987</v>
       </c>
       <c r="CT5">
-        <v>0.15746675200000004</v>
+        <v>0.15808287900000015</v>
       </c>
       <c r="CU5">
-        <v>5.4185071099999711E-2</v>
+        <v>5.4473591699999893E-2</v>
       </c>
       <c r="CV5">
-        <v>0.13218060799999978</v>
+        <v>0.13039472500000016</v>
       </c>
       <c r="CW5">
-        <v>0.20519655099999987</v>
+        <v>0.20165854299999961</v>
       </c>
       <c r="CX5">
-        <v>0.29311174500000048</v>
+        <v>0.29095957800000027</v>
       </c>
       <c r="CY5">
-        <v>0.36765543099999898</v>
+        <v>0.3689717650000004</v>
       </c>
       <c r="CZ5">
-        <v>0.39068396200000077</v>
+        <v>0.3939248729999994</v>
       </c>
       <c r="DA5">
-        <v>0.33555820600000036</v>
+        <v>0.33687066199999993</v>
       </c>
       <c r="DB5">
-        <v>0.26771007299999933</v>
+        <v>0.26811363100000035</v>
       </c>
       <c r="DC5">
-        <v>0.21059583999999995</v>
+        <v>0.20981275600000004</v>
       </c>
     </row>
     <row r="6" spans="1:107" x14ac:dyDescent="0.25">
@@ -9370,322 +9370,322 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>1.0723E-2</v>
+        <v>1.1174099999999999E-2</v>
       </c>
       <c r="C6">
-        <v>8.7557800000000005E-2</v>
+        <v>8.7376800000000004E-2</v>
       </c>
       <c r="D6">
-        <v>0.15548799999999999</v>
+        <v>0.15622179999999999</v>
       </c>
       <c r="E6">
-        <v>0.17169499999999999</v>
+        <v>0.17746200000000001</v>
       </c>
       <c r="F6">
-        <v>0.16005597500000002</v>
+        <v>0.17000209999999999</v>
       </c>
       <c r="G6">
-        <v>0.13955100000000001</v>
+        <v>0.150794025</v>
       </c>
       <c r="H6">
-        <v>0.110653</v>
+        <v>0.121611</v>
       </c>
       <c r="I6">
-        <v>7.7557399999999999E-2</v>
+        <v>8.6621699999999996E-2</v>
       </c>
       <c r="J6">
-        <v>6.9404822499999991E-2</v>
+        <v>7.0490225000000004E-2</v>
       </c>
       <c r="K6">
-        <v>0.24130674999999999</v>
+        <v>0.24318000000000001</v>
       </c>
       <c r="L6">
-        <v>0.23989199999999999</v>
+        <v>0.23734370000000002</v>
       </c>
       <c r="M6">
-        <v>0.183813</v>
+        <v>0.18570482500000002</v>
       </c>
       <c r="N6">
-        <v>0.15160599999999999</v>
+        <v>0.15436402500000002</v>
       </c>
       <c r="O6">
-        <v>0.12056934999999999</v>
+        <v>0.12231239999999999</v>
       </c>
       <c r="P6">
-        <v>8.5441100000000006E-2</v>
+        <v>8.6320174999999999E-2</v>
       </c>
       <c r="Q6">
-        <v>5.2861107499999997E-2</v>
+        <v>5.3568600000000001E-2</v>
       </c>
       <c r="R6">
-        <v>8.7571082499999994E-3</v>
+        <v>9.0820132499999998E-3</v>
       </c>
       <c r="S6">
-        <v>8.1074599999999997E-2</v>
+        <v>8.1286029999999995E-2</v>
       </c>
       <c r="T6">
-        <v>0.16755482499999999</v>
+        <v>0.16825000000000001</v>
       </c>
       <c r="U6">
-        <v>0.19454215</v>
+        <v>0.19845199999999999</v>
       </c>
       <c r="V6">
-        <v>0.18206700000000001</v>
+        <v>0.18920699999999999</v>
       </c>
       <c r="W6">
-        <v>0.154949</v>
+        <v>0.16248599999999999</v>
       </c>
       <c r="X6">
-        <v>0.12589504999999998</v>
+        <v>0.13243232499999999</v>
       </c>
       <c r="Y6">
-        <v>9.2656600000000006E-2</v>
+        <v>9.87952E-2</v>
       </c>
       <c r="Z6">
-        <v>5.95252E-2</v>
+        <v>6.4760100000000001E-2</v>
       </c>
       <c r="AA6">
-        <v>6.2107500000000003E-2</v>
+        <v>6.2592844999999994E-2</v>
       </c>
       <c r="AB6">
-        <v>0.243921</v>
+        <v>0.24504689999999998</v>
       </c>
       <c r="AC6">
-        <v>0.29651539999999998</v>
+        <v>0.29679100000000003</v>
       </c>
       <c r="AD6">
-        <v>0.23966599999999999</v>
+        <v>0.24054600000000001</v>
       </c>
       <c r="AE6">
-        <v>0.19344697499999999</v>
+        <v>0.19470499999999999</v>
       </c>
       <c r="AF6">
-        <v>0.15722164999999999</v>
+        <v>0.15795917499999998</v>
       </c>
       <c r="AG6">
-        <v>0.1184863</v>
+        <v>0.11835777500000001</v>
       </c>
       <c r="AH6">
-        <v>7.8330640000000007E-2</v>
+        <v>7.8138230000000003E-2</v>
       </c>
       <c r="AI6">
-        <v>4.5075299999999999E-2</v>
+        <v>4.4363899999999998E-2</v>
       </c>
       <c r="AJ6">
-        <v>8.3983884999999994E-3</v>
+        <v>8.5704600000000002E-3</v>
       </c>
       <c r="AK6">
-        <v>6.7923835000000002E-2</v>
+        <v>6.7271200000000003E-2</v>
       </c>
       <c r="AL6">
-        <v>0.15919939999999999</v>
+        <v>0.16075300000000001</v>
       </c>
       <c r="AM6">
-        <v>0.20504687500000002</v>
+        <v>0.20809492500000001</v>
       </c>
       <c r="AN6">
-        <v>0.19824117499999999</v>
+        <v>0.20299059999999999</v>
       </c>
       <c r="AO6">
-        <v>0.16800300000000001</v>
+        <v>0.17305000000000001</v>
       </c>
       <c r="AP6">
-        <v>0.13573499999999999</v>
+        <v>0.14011952499999999</v>
       </c>
       <c r="AQ6">
-        <v>0.10394289999999999</v>
+        <v>0.106986</v>
       </c>
       <c r="AR6">
-        <v>7.181709750000001E-2</v>
+        <v>7.38042E-2</v>
       </c>
       <c r="AS6">
-        <v>5.4736227499999998E-2</v>
+        <v>5.4369704999999997E-2</v>
       </c>
       <c r="AT6">
-        <v>0.22392200000000001</v>
+        <v>0.22331225000000002</v>
       </c>
       <c r="AU6">
-        <v>0.31642477500000005</v>
+        <v>0.31975900000000002</v>
       </c>
       <c r="AV6">
-        <v>0.29121202499999999</v>
+        <v>0.29339100000000001</v>
       </c>
       <c r="AW6">
-        <v>0.233071</v>
+        <v>0.23446800000000001</v>
       </c>
       <c r="AX6">
-        <v>0.187944</v>
+        <v>0.18890917499999998</v>
       </c>
       <c r="AY6">
-        <v>0.14677999999999999</v>
+        <v>0.14564099999999999</v>
       </c>
       <c r="AZ6">
-        <v>0.104099</v>
+        <v>0.10175427500000001</v>
       </c>
       <c r="BA6">
-        <v>6.4199645E-2</v>
+        <v>6.2188599999999997E-2</v>
       </c>
       <c r="BB6">
-        <v>1.29663E-2</v>
+        <v>1.3126282500000001E-2</v>
       </c>
       <c r="BC6">
-        <v>5.2947750000000002E-2</v>
+        <v>5.2292547499999995E-2</v>
       </c>
       <c r="BD6">
-        <v>0.13578077499999999</v>
+        <v>0.13582900000000001</v>
       </c>
       <c r="BE6">
-        <v>0.206032725</v>
+        <v>0.20817792500000001</v>
       </c>
       <c r="BF6">
-        <v>0.21659587500000002</v>
+        <v>0.220366175</v>
       </c>
       <c r="BG6">
-        <v>0.19267175</v>
+        <v>0.19587464999999998</v>
       </c>
       <c r="BH6">
-        <v>0.156229275</v>
+        <v>0.15845704999999999</v>
       </c>
       <c r="BI6">
-        <v>0.122202925</v>
+        <v>0.12273299999999999</v>
       </c>
       <c r="BJ6">
-        <v>9.0507099999999993E-2</v>
+        <v>8.9395199999999994E-2</v>
       </c>
       <c r="BK6">
-        <v>5.1442697500000002E-2</v>
+        <v>5.1120899999999997E-2</v>
       </c>
       <c r="BL6">
-        <v>0.190827</v>
+        <v>0.18792867500000002</v>
       </c>
       <c r="BM6">
-        <v>0.30184422500000002</v>
+        <v>0.30201899999999998</v>
       </c>
       <c r="BN6">
-        <v>0.34253800000000001</v>
+        <v>0.34599240000000003</v>
       </c>
       <c r="BO6">
-        <v>0.29638415000000001</v>
+        <v>0.298346</v>
       </c>
       <c r="BP6">
-        <v>0.23644427499999998</v>
+        <v>0.2378286</v>
       </c>
       <c r="BQ6">
-        <v>0.18747530000000001</v>
+        <v>0.186392</v>
       </c>
       <c r="BR6">
-        <v>0.14070042499999999</v>
+        <v>0.13855799999999999</v>
       </c>
       <c r="BS6">
-        <v>9.5212199999999997E-2</v>
+        <v>9.3079722500000003E-2</v>
       </c>
       <c r="BT6">
-        <v>2.44171925E-2</v>
+        <v>2.4644645E-2</v>
       </c>
       <c r="BU6">
-        <v>4.2976500000000001E-2</v>
+        <v>4.2492500000000002E-2</v>
       </c>
       <c r="BV6">
-        <v>0.100559</v>
+        <v>0.10044699999999999</v>
       </c>
       <c r="BW6">
-        <v>0.177262</v>
+        <v>0.17965100000000001</v>
       </c>
       <c r="BX6">
-        <v>0.22899095</v>
+        <v>0.23200799999999999</v>
       </c>
       <c r="BY6">
-        <v>0.22523199999999999</v>
+        <v>0.22851350000000001</v>
       </c>
       <c r="BZ6">
-        <v>0.19510967500000001</v>
+        <v>0.19694482500000002</v>
       </c>
       <c r="CA6">
-        <v>0.154972</v>
+        <v>0.15664060000000002</v>
       </c>
       <c r="CB6">
-        <v>0.11973085</v>
+        <v>0.11899800000000001</v>
       </c>
       <c r="CC6">
-        <v>5.6274499999999998E-2</v>
+        <v>5.6018600000000002E-2</v>
       </c>
       <c r="CD6">
-        <v>0.15121100000000001</v>
+        <v>0.14813897500000001</v>
       </c>
       <c r="CE6">
-        <v>0.25504045000000003</v>
+        <v>0.25194262499999998</v>
       </c>
       <c r="CF6">
-        <v>0.33816839999999998</v>
+        <v>0.33805649999999998</v>
       </c>
       <c r="CG6">
-        <v>0.36622900000000003</v>
+        <v>0.36942999999999998</v>
       </c>
       <c r="CH6">
-        <v>0.31473400000000001</v>
+        <v>0.317589275</v>
       </c>
       <c r="CI6">
-        <v>0.25047914999999998</v>
+        <v>0.25112709999999999</v>
       </c>
       <c r="CJ6">
-        <v>0.19570694999999999</v>
+        <v>0.19419400000000001</v>
       </c>
       <c r="CK6">
-        <v>0.145005</v>
+        <v>0.14263999999999999</v>
       </c>
       <c r="CL6">
-        <v>2.84418E-2</v>
+        <v>2.8604894999999998E-2</v>
       </c>
       <c r="CM6">
-        <v>4.1586524999999999E-2</v>
+        <v>4.1162955000000001E-2</v>
       </c>
       <c r="CN6">
-        <v>7.0877399999999993E-2</v>
+        <v>7.0173252499999991E-2</v>
       </c>
       <c r="CO6">
-        <v>0.12900500000000001</v>
+        <v>0.13032820000000001</v>
       </c>
       <c r="CP6">
-        <v>0.19595199999999999</v>
+        <v>0.19876950000000002</v>
       </c>
       <c r="CQ6">
-        <v>0.23621250000000002</v>
+        <v>0.23894465000000001</v>
       </c>
       <c r="CR6">
-        <v>0.22592100000000001</v>
+        <v>0.22839499999999999</v>
       </c>
       <c r="CS6">
-        <v>0.193262925</v>
+        <v>0.194493</v>
       </c>
       <c r="CT6">
-        <v>0.15248420000000001</v>
+        <v>0.15360342499999999</v>
       </c>
       <c r="CU6">
-        <v>5.1980100000000001E-2</v>
+        <v>5.1968455000000004E-2</v>
       </c>
       <c r="CV6">
-        <v>0.12689365</v>
+        <v>0.123436225</v>
       </c>
       <c r="CW6">
-        <v>0.197746425</v>
+        <v>0.19290017499999998</v>
       </c>
       <c r="CX6">
-        <v>0.28447964999999997</v>
+        <v>0.28189199999999998</v>
       </c>
       <c r="CY6">
-        <v>0.35804644999999996</v>
+        <v>0.358103</v>
       </c>
       <c r="CZ6">
-        <v>0.37966735000000001</v>
+        <v>0.38152799999999998</v>
       </c>
       <c r="DA6">
-        <v>0.32469999999999999</v>
+        <v>0.326963</v>
       </c>
       <c r="DB6">
-        <v>0.25781575000000001</v>
+        <v>0.25825549999999997</v>
       </c>
       <c r="DC6">
-        <v>0.20050669999999998</v>
+        <v>0.19875599999999999</v>
       </c>
     </row>
     <row r="7" spans="1:107" x14ac:dyDescent="0.25">
@@ -9693,322 +9693,322 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>1.3979859999999998E-2</v>
+        <v>1.4406499999999999E-2</v>
       </c>
       <c r="C7">
-        <v>0.1034939</v>
+        <v>0.10410084999999999</v>
       </c>
       <c r="D7">
-        <v>0.178367</v>
+        <v>0.17921500000000001</v>
       </c>
       <c r="E7">
-        <v>0.19820399999999999</v>
+        <v>0.20191964999999998</v>
       </c>
       <c r="F7">
-        <v>0.19032299999999999</v>
+        <v>0.19716919999999999</v>
       </c>
       <c r="G7">
-        <v>0.16969600000000001</v>
+        <v>0.17690757500000001</v>
       </c>
       <c r="H7">
-        <v>0.139876</v>
+        <v>0.14613809999999999</v>
       </c>
       <c r="I7">
-        <v>0.10295600000000001</v>
+        <v>0.10799212499999999</v>
       </c>
       <c r="J7">
-        <v>8.3139237500000004E-2</v>
+        <v>8.4090600000000001E-2</v>
       </c>
       <c r="K7">
-        <v>0.26770512500000004</v>
+        <v>0.26775300000000002</v>
       </c>
       <c r="L7">
-        <v>0.26780199999999998</v>
+        <v>0.26448899999999997</v>
       </c>
       <c r="M7">
-        <v>0.20856769999999999</v>
+        <v>0.20588999999999999</v>
       </c>
       <c r="N7">
-        <v>0.17274820000000002</v>
+        <v>0.17110700000000001</v>
       </c>
       <c r="O7">
-        <v>0.140789</v>
+        <v>0.137362175</v>
       </c>
       <c r="P7">
-        <v>0.103495</v>
+        <v>0.10045999999999999</v>
       </c>
       <c r="Q7">
-        <v>6.7127507500000003E-2</v>
+        <v>6.5228427499999991E-2</v>
       </c>
       <c r="R7">
-        <v>1.1260715000000001E-2</v>
+        <v>1.1584499999999999E-2</v>
       </c>
       <c r="S7">
-        <v>9.472014749999999E-2</v>
+        <v>9.5901092499999993E-2</v>
       </c>
       <c r="T7">
-        <v>0.189331</v>
+        <v>0.190194</v>
       </c>
       <c r="U7">
-        <v>0.218501</v>
+        <v>0.22021004999999999</v>
       </c>
       <c r="V7">
-        <v>0.20538210000000001</v>
+        <v>0.21021000000000001</v>
       </c>
       <c r="W7">
-        <v>0.17686399999999999</v>
+        <v>0.18381547500000001</v>
       </c>
       <c r="X7">
-        <v>0.14607999999999999</v>
+        <v>0.15296199999999999</v>
       </c>
       <c r="Y7">
-        <v>0.11176</v>
+        <v>0.11734</v>
       </c>
       <c r="Z7">
-        <v>7.6178300000000004E-2</v>
+        <v>7.9897300000000004E-2</v>
       </c>
       <c r="AA7">
-        <v>7.3292952499999994E-2</v>
+        <v>7.3565900000000004E-2</v>
       </c>
       <c r="AB7">
-        <v>0.26611499999999999</v>
+        <v>0.26532577499999999</v>
       </c>
       <c r="AC7">
-        <v>0.31920969999999999</v>
+        <v>0.31881635000000003</v>
       </c>
       <c r="AD7">
-        <v>0.26154757499999998</v>
+        <v>0.26003987499999998</v>
       </c>
       <c r="AE7">
-        <v>0.21177599999999999</v>
+        <v>0.21155237499999999</v>
       </c>
       <c r="AF7">
-        <v>0.1739937</v>
+        <v>0.17320822499999999</v>
       </c>
       <c r="AG7">
-        <v>0.13503762499999999</v>
+        <v>0.13192654999999998</v>
       </c>
       <c r="AH7">
-        <v>9.3513799999999994E-2</v>
+        <v>9.0787762499999994E-2</v>
       </c>
       <c r="AI7">
-        <v>5.6868299999999997E-2</v>
+        <v>5.5166300000000001E-2</v>
       </c>
       <c r="AJ7">
-        <v>1.0633872500000001E-2</v>
+        <v>1.0872E-2</v>
       </c>
       <c r="AK7">
-        <v>7.9196979999999986E-2</v>
+        <v>7.9076599999999997E-2</v>
       </c>
       <c r="AL7">
-        <v>0.18041639999999998</v>
+        <v>0.18057657500000002</v>
       </c>
       <c r="AM7">
-        <v>0.22720699999999999</v>
+        <v>0.22774997499999999</v>
       </c>
       <c r="AN7">
-        <v>0.21709800000000001</v>
+        <v>0.22004499999999999</v>
       </c>
       <c r="AO7">
-        <v>0.18381400000000001</v>
+        <v>0.18854399999999999</v>
       </c>
       <c r="AP7">
-        <v>0.150346175</v>
+        <v>0.154917</v>
       </c>
       <c r="AQ7">
-        <v>0.117891</v>
+        <v>0.12123979999999999</v>
       </c>
       <c r="AR7">
-        <v>8.4771927499999997E-2</v>
+        <v>8.6524457499999999E-2</v>
       </c>
       <c r="AS7">
-        <v>6.3961309999999993E-2</v>
+        <v>6.37889975E-2</v>
       </c>
       <c r="AT7">
-        <v>0.24283352499999999</v>
+        <v>0.240859875</v>
       </c>
       <c r="AU7">
-        <v>0.33893600000000002</v>
+        <v>0.33783200000000002</v>
       </c>
       <c r="AV7">
-        <v>0.311776</v>
+        <v>0.31106299999999998</v>
       </c>
       <c r="AW7">
-        <v>0.25305499999999997</v>
+        <v>0.24987774999999998</v>
       </c>
       <c r="AX7">
-        <v>0.204986</v>
+        <v>0.20525260000000001</v>
       </c>
       <c r="AY7">
-        <v>0.16250899999999999</v>
+        <v>0.16180129999999998</v>
       </c>
       <c r="AZ7">
-        <v>0.1187719</v>
+        <v>0.11641595</v>
       </c>
       <c r="BA7">
-        <v>7.7412869999999995E-2</v>
+        <v>7.4605297499999987E-2</v>
       </c>
       <c r="BB7">
-        <v>1.5198700000000001E-2</v>
+        <v>1.5415099999999999E-2</v>
       </c>
       <c r="BC7">
-        <v>6.1880900000000003E-2</v>
+        <v>6.0801399999999999E-2</v>
       </c>
       <c r="BD7">
-        <v>0.15434052500000001</v>
+        <v>0.153142</v>
       </c>
       <c r="BE7">
-        <v>0.226218</v>
+        <v>0.22754754999999999</v>
       </c>
       <c r="BF7">
-        <v>0.233791</v>
+        <v>0.23706145000000001</v>
       </c>
       <c r="BG7">
-        <v>0.20587692499999999</v>
+        <v>0.20954300000000001</v>
       </c>
       <c r="BH7">
-        <v>0.16822999999999999</v>
+        <v>0.16894100000000001</v>
       </c>
       <c r="BI7">
-        <v>0.133885</v>
+        <v>0.133913</v>
       </c>
       <c r="BJ7">
-        <v>0.102023</v>
+        <v>0.101256575</v>
       </c>
       <c r="BK7">
-        <v>5.92437325E-2</v>
+        <v>5.8814900000000003E-2</v>
       </c>
       <c r="BL7">
-        <v>0.20730627499999998</v>
+        <v>0.20458699999999999</v>
       </c>
       <c r="BM7">
-        <v>0.32187700000000002</v>
+        <v>0.32079099999999999</v>
       </c>
       <c r="BN7">
-        <v>0.36365399999999998</v>
+        <v>0.36363855</v>
       </c>
       <c r="BO7">
-        <v>0.317467</v>
+        <v>0.31519934999999999</v>
       </c>
       <c r="BP7">
-        <v>0.256158</v>
+        <v>0.25416699999999998</v>
       </c>
       <c r="BQ7">
-        <v>0.20475599999999999</v>
+        <v>0.20408899999999999</v>
       </c>
       <c r="BR7">
-        <v>0.15653265</v>
+        <v>0.154779325</v>
       </c>
       <c r="BS7">
-        <v>0.110709525</v>
+        <v>0.10711</v>
       </c>
       <c r="BT7">
-        <v>2.6317500000000001E-2</v>
+        <v>2.6435E-2</v>
       </c>
       <c r="BU7">
-        <v>4.9566934999999999E-2</v>
+        <v>4.8529094999999994E-2</v>
       </c>
       <c r="BV7">
-        <v>0.115658</v>
+        <v>0.11312367499999999</v>
       </c>
       <c r="BW7">
-        <v>0.19695799999999999</v>
+        <v>0.196828525</v>
       </c>
       <c r="BX7">
-        <v>0.24651999999999999</v>
+        <v>0.249819975</v>
       </c>
       <c r="BY7">
-        <v>0.23944399999999999</v>
+        <v>0.24478254999999999</v>
       </c>
       <c r="BZ7">
-        <v>0.20750199999999999</v>
+        <v>0.209534475</v>
       </c>
       <c r="CA7">
-        <v>0.16612499999999999</v>
+        <v>0.16605800000000001</v>
       </c>
       <c r="CB7">
-        <v>0.13092720000000002</v>
+        <v>0.12978487499999999</v>
       </c>
       <c r="CC7">
-        <v>6.2814700000000001E-2</v>
+        <v>6.2133000000000001E-2</v>
       </c>
       <c r="CD7">
-        <v>0.16625000000000001</v>
+        <v>0.162421175</v>
       </c>
       <c r="CE7">
-        <v>0.27251500000000001</v>
+        <v>0.26984007500000001</v>
       </c>
       <c r="CF7">
-        <v>0.35859437500000002</v>
+        <v>0.358732</v>
       </c>
       <c r="CG7">
-        <v>0.38794055</v>
+        <v>0.39069700000000002</v>
       </c>
       <c r="CH7">
-        <v>0.34024399999999999</v>
+        <v>0.33572400000000002</v>
       </c>
       <c r="CI7">
-        <v>0.27144360000000001</v>
+        <v>0.2689666</v>
       </c>
       <c r="CJ7">
-        <v>0.21479100000000001</v>
+        <v>0.21328549999999999</v>
       </c>
       <c r="CK7">
-        <v>0.16283265</v>
+        <v>0.16012799999999999</v>
       </c>
       <c r="CL7">
-        <v>3.0049099999999999E-2</v>
+        <v>3.0162999999999999E-2</v>
       </c>
       <c r="CM7">
-        <v>4.5196600000000003E-2</v>
+        <v>4.5016800000000003E-2</v>
       </c>
       <c r="CN7">
-        <v>8.0908999999999995E-2</v>
+        <v>7.9544727499999995E-2</v>
       </c>
       <c r="CO7">
-        <v>0.14645434999999998</v>
+        <v>0.14498025</v>
       </c>
       <c r="CP7">
-        <v>0.21446000000000001</v>
+        <v>0.21565300000000001</v>
       </c>
       <c r="CQ7">
-        <v>0.25108965</v>
+        <v>0.255662</v>
       </c>
       <c r="CR7">
-        <v>0.239401</v>
+        <v>0.243992925</v>
       </c>
       <c r="CS7">
-        <v>0.20536925</v>
+        <v>0.20607</v>
       </c>
       <c r="CT7">
-        <v>0.163387</v>
+        <v>0.162191</v>
       </c>
       <c r="CU7">
-        <v>5.67591E-2</v>
+        <v>5.70453E-2</v>
       </c>
       <c r="CV7">
-        <v>0.13970217499999998</v>
+        <v>0.13780500000000001</v>
       </c>
       <c r="CW7">
-        <v>0.21524299999999999</v>
+        <v>0.210783</v>
       </c>
       <c r="CX7">
-        <v>0.30335899999999999</v>
+        <v>0.30108200000000002</v>
       </c>
       <c r="CY7">
-        <v>0.37955</v>
+        <v>0.380936</v>
       </c>
       <c r="CZ7">
-        <v>0.403055</v>
+        <v>0.40497495</v>
       </c>
       <c r="DA7">
-        <v>0.35151199999999999</v>
+        <v>0.347609</v>
       </c>
       <c r="DB7">
-        <v>0.27996492499999998</v>
+        <v>0.27671899999999999</v>
       </c>
       <c r="DC7">
-        <v>0.22046499999999999</v>
+        <v>0.218614</v>
       </c>
     </row>
   </sheetData>
@@ -11000,322 +11000,322 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>1.2902595500000016E-2</v>
+        <v>1.3335662899999996E-2</v>
       </c>
       <c r="C5">
-        <v>9.600264740000003E-2</v>
+        <v>9.5492582100000098E-2</v>
       </c>
       <c r="D5">
-        <v>0.16507378199999995</v>
+        <v>0.16491113000000018</v>
       </c>
       <c r="E5">
-        <v>0.18241058199999996</v>
+        <v>0.18851204000000016</v>
       </c>
       <c r="F5">
-        <v>0.17277386600000022</v>
+        <v>0.18382793700000022</v>
       </c>
       <c r="G5">
-        <v>0.15292886599999991</v>
+        <v>0.16481992399999976</v>
       </c>
       <c r="H5">
-        <v>0.12390827300000011</v>
+        <v>0.13485192199999968</v>
       </c>
       <c r="I5">
-        <v>8.8527025999999912E-2</v>
+        <v>9.746565270000021E-2</v>
       </c>
       <c r="J5">
-        <v>7.7661587299999973E-2</v>
+        <v>7.9425620199999811E-2</v>
       </c>
       <c r="K5">
-        <v>0.25632468900000016</v>
+        <v>0.25646782799999968</v>
       </c>
       <c r="L5">
-        <v>0.25293162599999996</v>
+        <v>0.25160812799999971</v>
       </c>
       <c r="M5">
-        <v>0.19629791200000038</v>
+        <v>0.19775361500000019</v>
       </c>
       <c r="N5">
-        <v>0.16265669999999982</v>
+        <v>0.16399958099999995</v>
       </c>
       <c r="O5">
-        <v>0.130062331</v>
+        <v>0.12945616999999968</v>
       </c>
       <c r="P5">
-        <v>9.2761575799999899E-2</v>
+        <v>9.1137570199999962E-2</v>
       </c>
       <c r="Q5">
-        <v>5.7893477199999981E-2</v>
+        <v>5.6384499499999984E-2</v>
       </c>
       <c r="R5">
-        <v>1.0483775500000011E-2</v>
+        <v>1.0780603850000018E-2</v>
       </c>
       <c r="S5">
-        <v>8.9038033000000086E-2</v>
+        <v>8.8731249699999876E-2</v>
       </c>
       <c r="T5">
-        <v>0.17839636900000025</v>
+        <v>0.17768832000000026</v>
       </c>
       <c r="U5">
-        <v>0.20443259700000033</v>
+        <v>0.20718139599999941</v>
       </c>
       <c r="V5">
-        <v>0.19194312700000024</v>
+        <v>0.19903710199999947</v>
       </c>
       <c r="W5">
-        <v>0.16519559400000006</v>
+        <v>0.1738538170000001</v>
       </c>
       <c r="X5">
-        <v>0.13539083700000004</v>
+        <v>0.14358590000000004</v>
       </c>
       <c r="Y5">
-        <v>0.10150858979999995</v>
+        <v>0.10842249869999979</v>
       </c>
       <c r="Z5">
-        <v>6.7088531100000057E-2</v>
+        <v>7.221087400000005E-2</v>
       </c>
       <c r="AA5">
-        <v>6.9047646699999785E-2</v>
+        <v>7.0313098800000126E-2</v>
       </c>
       <c r="AB5">
-        <v>0.25757386799999993</v>
+        <v>0.2577566879999994</v>
       </c>
       <c r="AC5">
-        <v>0.30905263299999924</v>
+        <v>0.3077056290000002</v>
       </c>
       <c r="AD5">
-        <v>0.25072559399999983</v>
+        <v>0.25010961099999973</v>
       </c>
       <c r="AE5">
-        <v>0.20262223799999993</v>
+        <v>0.20399138300000005</v>
       </c>
       <c r="AF5">
-        <v>0.16576875299999974</v>
+        <v>0.16613117499999999</v>
       </c>
       <c r="AG5">
-        <v>0.12568582699999992</v>
+        <v>0.12467830799999992</v>
       </c>
       <c r="AH5">
-        <v>8.459740699999975E-2</v>
+        <v>8.3175363300000055E-2</v>
       </c>
       <c r="AI5">
-        <v>4.9365666099999934E-2</v>
+        <v>4.8265084999999992E-2</v>
       </c>
       <c r="AJ5">
-        <v>9.865715560000014E-3</v>
+        <v>9.9948657100000053E-3</v>
       </c>
       <c r="AK5">
-        <v>7.4612747700000009E-2</v>
+        <v>7.4169574200000032E-2</v>
       </c>
       <c r="AL5">
-        <v>0.1710693599999997</v>
+        <v>0.17020493600000061</v>
       </c>
       <c r="AM5">
-        <v>0.21541370999999984</v>
+        <v>0.21638510799999966</v>
       </c>
       <c r="AN5">
-        <v>0.20668392599999996</v>
+        <v>0.21033946199999917</v>
       </c>
       <c r="AO5">
-        <v>0.17576672599999979</v>
+        <v>0.18093893499999975</v>
       </c>
       <c r="AP5">
-        <v>0.1431651510000001</v>
+        <v>0.14815613300000002</v>
       </c>
       <c r="AQ5">
-        <v>0.11075738599999986</v>
+        <v>0.11490074000000017</v>
       </c>
       <c r="AR5">
-        <v>7.7520230499999815E-2</v>
+        <v>8.0618493700000016E-2</v>
       </c>
       <c r="AS5">
-        <v>6.0245951800000037E-2</v>
+        <v>6.0902879899999991E-2</v>
       </c>
       <c r="AT5">
-        <v>0.23530667500000016</v>
+        <v>0.23468841799999993</v>
       </c>
       <c r="AU5">
-        <v>0.32999064000000028</v>
+        <v>0.3287124429999998</v>
       </c>
       <c r="AV5">
-        <v>0.3023903910000002</v>
+        <v>0.30046172900000034</v>
       </c>
       <c r="AW5">
-        <v>0.24179426499999959</v>
+        <v>0.24165656199999949</v>
       </c>
       <c r="AX5">
-        <v>0.19651881499999971</v>
+        <v>0.19710479500000036</v>
       </c>
       <c r="AY5">
-        <v>0.15448694899999976</v>
+        <v>0.15399982200000004</v>
       </c>
       <c r="AZ5">
-        <v>0.11048762689999984</v>
+        <v>0.10915920399999982</v>
       </c>
       <c r="BA5">
-        <v>6.9654105799999894E-2</v>
+        <v>6.8268376900000094E-2</v>
       </c>
       <c r="BB5">
-        <v>1.4407409300000028E-2</v>
+        <v>1.4541266800000013E-2</v>
       </c>
       <c r="BC5">
-        <v>5.8183462799999926E-2</v>
+        <v>5.7531525300000115E-2</v>
       </c>
       <c r="BD5">
-        <v>0.14583636000000039</v>
+        <v>0.14474145500000027</v>
       </c>
       <c r="BE5">
-        <v>0.21704046800000043</v>
+        <v>0.21706538100000003</v>
       </c>
       <c r="BF5">
-        <v>0.22547804900000015</v>
+        <v>0.22676475199999982</v>
       </c>
       <c r="BG5">
-        <v>0.1994583490000004</v>
+        <v>0.20152670300000025</v>
       </c>
       <c r="BH5">
-        <v>0.16188815600000014</v>
+        <v>0.16412745299999995</v>
       </c>
       <c r="BI5">
-        <v>0.12790802600000051</v>
+        <v>0.12961097700000024</v>
       </c>
       <c r="BJ5">
-        <v>9.5675046800000163E-2</v>
+        <v>9.6753474099999917E-2</v>
       </c>
       <c r="BK5">
-        <v>5.5629287500000069E-2</v>
+        <v>5.5980934199999874E-2</v>
       </c>
       <c r="BL5">
-        <v>0.20015296499999952</v>
+        <v>0.19830278799999984</v>
       </c>
       <c r="BM5">
-        <v>0.31441025300000053</v>
+        <v>0.31222519000000004</v>
       </c>
       <c r="BN5">
-        <v>0.35589101400000095</v>
+        <v>0.35384322000000001</v>
       </c>
       <c r="BO5">
-        <v>0.30711891099999999</v>
+        <v>0.30481634800000057</v>
       </c>
       <c r="BP5">
-        <v>0.24566090399999957</v>
+        <v>0.24508226199999963</v>
       </c>
       <c r="BQ5">
-        <v>0.19601362899999988</v>
+        <v>0.19567233100000017</v>
       </c>
       <c r="BR5">
-        <v>0.14887458300000003</v>
+        <v>0.14758027000000018</v>
       </c>
       <c r="BS5">
-        <v>0.10252435790000024</v>
+        <v>0.1006330716999999</v>
       </c>
       <c r="BT5">
-        <v>2.5456758200000009E-2</v>
+        <v>2.5724400299999981E-2</v>
       </c>
       <c r="BU5">
-        <v>4.6816844899999988E-2</v>
+        <v>4.6269733999999889E-2</v>
       </c>
       <c r="BV5">
-        <v>0.10833716169999998</v>
+        <v>0.10701324569999977</v>
       </c>
       <c r="BW5">
-        <v>0.18770542499999984</v>
+        <v>0.187443424</v>
       </c>
       <c r="BX5">
-        <v>0.23866823400000017</v>
+        <v>0.23904052299999995</v>
       </c>
       <c r="BY5">
-        <v>0.23294847100000016</v>
+        <v>0.23357430199999993</v>
       </c>
       <c r="BZ5">
-        <v>0.20087193600000039</v>
+        <v>0.20157939799999988</v>
       </c>
       <c r="CA5">
-        <v>0.1605946540000002</v>
+        <v>0.16124829199999996</v>
       </c>
       <c r="CB5">
-        <v>0.12542822300000006</v>
+        <v>0.12563504500000017</v>
       </c>
       <c r="CC5">
-        <v>5.8769334800000156E-2</v>
+        <v>5.9187595499999947E-2</v>
       </c>
       <c r="CD5">
-        <v>0.15782917499999996</v>
+        <v>0.15554252700000024</v>
       </c>
       <c r="CE5">
-        <v>0.26471116200000022</v>
+        <v>0.26117940700000053</v>
       </c>
       <c r="CF5">
-        <v>0.35115473900000077</v>
+        <v>0.34830004500000061</v>
       </c>
       <c r="CG5">
-        <v>0.38105848299999934</v>
+        <v>0.37853840399999944</v>
       </c>
       <c r="CH5">
-        <v>0.32700015200000021</v>
+        <v>0.32420062200000016</v>
       </c>
       <c r="CI5">
-        <v>0.26072421999999973</v>
+        <v>0.25944248500000033</v>
       </c>
       <c r="CJ5">
-        <v>0.20550578500000014</v>
+        <v>0.2044607600000003</v>
       </c>
       <c r="CK5">
-        <v>0.15463815899999978</v>
+        <v>0.15268222200000006</v>
       </c>
       <c r="CL5">
-        <v>2.9311210200000062E-2</v>
+        <v>2.9513196400000035E-2</v>
       </c>
       <c r="CM5">
-        <v>4.3679648999999918E-2</v>
+        <v>4.3563506299999999E-2</v>
       </c>
       <c r="CN5">
-        <v>7.5941073400000086E-2</v>
+        <v>7.4850588499999995E-2</v>
       </c>
       <c r="CO5">
-        <v>0.13730109700000007</v>
+        <v>0.13669959700000042</v>
       </c>
       <c r="CP5">
-        <v>0.20516229299999986</v>
+        <v>0.20558682299999956</v>
       </c>
       <c r="CQ5">
-        <v>0.24427643800000032</v>
+        <v>0.24449710099999958</v>
       </c>
       <c r="CR5">
-        <v>0.2328379729999995</v>
+        <v>0.23289966000000017</v>
       </c>
       <c r="CS5">
-        <v>0.19866628600000052</v>
+        <v>0.19863140399999987</v>
       </c>
       <c r="CT5">
-        <v>0.15777542100000005</v>
+        <v>0.15765358299999993</v>
       </c>
       <c r="CU5">
-        <v>5.3345043199999963E-2</v>
+        <v>5.3711824700000174E-2</v>
       </c>
       <c r="CV5">
-        <v>0.12993944000000024</v>
+        <v>0.12829848500000024</v>
       </c>
       <c r="CW5">
-        <v>0.20427799500000007</v>
+        <v>0.20048670199999985</v>
       </c>
       <c r="CX5">
-        <v>0.29493041999999958</v>
+        <v>0.2909190020000007</v>
       </c>
       <c r="CY5">
-        <v>0.37202807399999949</v>
+        <v>0.36885117499999942</v>
       </c>
       <c r="CZ5">
-        <v>0.3950910650000008</v>
+        <v>0.39224052400000009</v>
       </c>
       <c r="DA5">
-        <v>0.33785869500000026</v>
+        <v>0.33472571499999965</v>
       </c>
       <c r="DB5">
-        <v>0.26879282300000051</v>
+        <v>0.26711582300000064</v>
       </c>
       <c r="DC5">
-        <v>0.21113514700000005</v>
+        <v>0.20970033299999932</v>
       </c>
     </row>
     <row r="6" spans="1:107" x14ac:dyDescent="0.25">
@@ -11323,322 +11323,322 @@
         <v>15</v>
       </c>
       <c r="B6">
-        <v>1.1253300000000001E-2</v>
+        <v>1.16866825E-2</v>
       </c>
       <c r="C6">
-        <v>8.8783097500000005E-2</v>
+        <v>8.7270799999999996E-2</v>
       </c>
       <c r="D6">
-        <v>0.15506737499999998</v>
+        <v>0.15368809999999999</v>
       </c>
       <c r="E6">
-        <v>0.168521</v>
+        <v>0.17668050000000002</v>
       </c>
       <c r="F6">
-        <v>0.153639</v>
+        <v>0.16908287499999999</v>
       </c>
       <c r="G6">
-        <v>0.13290299999999999</v>
+        <v>0.14929534999999999</v>
       </c>
       <c r="H6">
-        <v>0.105452</v>
+        <v>0.11999620000000001</v>
       </c>
       <c r="I6">
-        <v>7.3360400000000006E-2</v>
+        <v>8.4364947500000009E-2</v>
       </c>
       <c r="J6">
-        <v>7.1199187499999997E-2</v>
+        <v>7.3313890000000007E-2</v>
       </c>
       <c r="K6">
-        <v>0.24288799999999999</v>
+        <v>0.244949</v>
       </c>
       <c r="L6">
-        <v>0.239097475</v>
+        <v>0.24042164999999999</v>
       </c>
       <c r="M6">
-        <v>0.185891</v>
+        <v>0.186893</v>
       </c>
       <c r="N6">
-        <v>0.15325845000000002</v>
+        <v>0.15471427499999998</v>
       </c>
       <c r="O6">
-        <v>0.12177</v>
+        <v>0.120314</v>
       </c>
       <c r="P6">
-        <v>8.5559597500000001E-2</v>
+        <v>8.3490400000000006E-2</v>
       </c>
       <c r="Q6">
-        <v>5.18758E-2</v>
+        <v>5.0465000000000003E-2</v>
       </c>
       <c r="R6">
-        <v>9.2224899999999999E-3</v>
+        <v>9.5388364999999999E-3</v>
       </c>
       <c r="S6">
-        <v>8.2541765000000003E-2</v>
+        <v>8.19323E-2</v>
       </c>
       <c r="T6">
-        <v>0.169043675</v>
+        <v>0.16622400000000001</v>
       </c>
       <c r="U6">
-        <v>0.194635</v>
+        <v>0.19760355000000002</v>
       </c>
       <c r="V6">
-        <v>0.178704</v>
+        <v>0.18890119999999999</v>
       </c>
       <c r="W6">
-        <v>0.151034</v>
+        <v>0.16275972499999999</v>
       </c>
       <c r="X6">
-        <v>0.12239700000000001</v>
+        <v>0.132613225</v>
       </c>
       <c r="Y6">
-        <v>9.0471099999999999E-2</v>
+        <v>9.793002499999999E-2</v>
       </c>
       <c r="Z6">
-        <v>5.8700599999999999E-2</v>
+        <v>6.3762365000000001E-2</v>
       </c>
       <c r="AA6">
-        <v>6.3621700000000003E-2</v>
+        <v>6.5441207500000001E-2</v>
       </c>
       <c r="AB6">
-        <v>0.24657499999999999</v>
+        <v>0.24723300000000001</v>
       </c>
       <c r="AC6">
-        <v>0.29719665000000001</v>
+        <v>0.29623699999999997</v>
       </c>
       <c r="AD6">
-        <v>0.24027964999999998</v>
+        <v>0.23949300000000001</v>
       </c>
       <c r="AE6">
-        <v>0.193943</v>
+        <v>0.194719</v>
       </c>
       <c r="AF6">
-        <v>0.157829725</v>
+        <v>0.15815000000000001</v>
       </c>
       <c r="AG6">
-        <v>0.118430825</v>
+        <v>0.116762</v>
       </c>
       <c r="AH6">
-        <v>7.7775899999999995E-2</v>
+        <v>7.66738E-2</v>
       </c>
       <c r="AI6">
-        <v>4.4507762499999999E-2</v>
+        <v>4.3246399999999997E-2</v>
       </c>
       <c r="AJ6">
-        <v>8.7076800000000006E-3</v>
+        <v>8.8271917499999995E-3</v>
       </c>
       <c r="AK6">
-        <v>6.9585965E-2</v>
+        <v>6.8557900000000005E-2</v>
       </c>
       <c r="AL6">
-        <v>0.162175875</v>
+        <v>0.15929699999999999</v>
       </c>
       <c r="AM6">
-        <v>0.207007525</v>
+        <v>0.20552100000000001</v>
       </c>
       <c r="AN6">
-        <v>0.19772899999999999</v>
+        <v>0.202293</v>
       </c>
       <c r="AO6">
-        <v>0.166603</v>
+        <v>0.17341799999999999</v>
       </c>
       <c r="AP6">
-        <v>0.135295</v>
+        <v>0.140567</v>
       </c>
       <c r="AQ6">
-        <v>0.104271</v>
+        <v>0.10752299999999999</v>
       </c>
       <c r="AR6">
-        <v>7.1863492500000001E-2</v>
+        <v>7.4227004999999999E-2</v>
       </c>
       <c r="AS6">
-        <v>5.5445599999999998E-2</v>
+        <v>5.7072199999999997E-2</v>
       </c>
       <c r="AT6">
-        <v>0.22530952500000001</v>
+        <v>0.22631200000000001</v>
       </c>
       <c r="AU6">
-        <v>0.318797</v>
+        <v>0.31722699999999998</v>
       </c>
       <c r="AV6">
-        <v>0.29213742500000001</v>
+        <v>0.29082999999999998</v>
       </c>
       <c r="AW6">
-        <v>0.23277450000000002</v>
+        <v>0.23255600000000001</v>
       </c>
       <c r="AX6">
-        <v>0.188337</v>
+        <v>0.18909599999999999</v>
       </c>
       <c r="AY6">
-        <v>0.1473554</v>
+        <v>0.14668</v>
       </c>
       <c r="AZ6">
-        <v>0.1036299</v>
+        <v>0.102326525</v>
       </c>
       <c r="BA6">
-        <v>6.3950400000000004E-2</v>
+        <v>6.2553065000000005E-2</v>
       </c>
       <c r="BB6">
-        <v>1.3289805E-2</v>
+        <v>1.3263799999999999E-2</v>
       </c>
       <c r="BC6">
-        <v>5.4362515E-2</v>
+        <v>5.2954500000000002E-2</v>
       </c>
       <c r="BD6">
-        <v>0.137545</v>
+        <v>0.135101</v>
       </c>
       <c r="BE6">
-        <v>0.208472875</v>
+        <v>0.207122</v>
       </c>
       <c r="BF6">
-        <v>0.2177133</v>
+        <v>0.21851799999999999</v>
       </c>
       <c r="BG6">
-        <v>0.19334499999999999</v>
+        <v>0.19537599999999999</v>
       </c>
       <c r="BH6">
-        <v>0.15677137499999999</v>
+        <v>0.15857099999999999</v>
       </c>
       <c r="BI6">
-        <v>0.122595475</v>
+        <v>0.12482500000000001</v>
       </c>
       <c r="BJ6">
-        <v>9.0991900000000001E-2</v>
+        <v>9.1979980000000003E-2</v>
       </c>
       <c r="BK6">
-        <v>5.1561000000000003E-2</v>
+        <v>5.2704139999999997E-2</v>
       </c>
       <c r="BL6">
-        <v>0.191161</v>
+        <v>0.190412</v>
       </c>
       <c r="BM6">
-        <v>0.30439045000000003</v>
+        <v>0.30309599999999998</v>
       </c>
       <c r="BN6">
-        <v>0.344316925</v>
+        <v>0.34331899999999999</v>
       </c>
       <c r="BO6">
-        <v>0.29797570000000001</v>
+        <v>0.296149</v>
       </c>
       <c r="BP6">
-        <v>0.23705999999999999</v>
+        <v>0.23639235</v>
       </c>
       <c r="BQ6">
-        <v>0.188080475</v>
+        <v>0.18801852499999999</v>
       </c>
       <c r="BR6">
-        <v>0.14195085000000002</v>
+        <v>0.14052249999999999</v>
       </c>
       <c r="BS6">
-        <v>9.6077399999999993E-2</v>
+        <v>9.4270400000000004E-2</v>
       </c>
       <c r="BT6">
-        <v>2.4508465E-2</v>
+        <v>2.47502E-2</v>
       </c>
       <c r="BU6">
-        <v>4.3918177499999995E-2</v>
+        <v>4.3119797500000001E-2</v>
       </c>
       <c r="BV6">
-        <v>0.10165815</v>
+        <v>9.9797899999999995E-2</v>
       </c>
       <c r="BW6">
-        <v>0.17895900000000001</v>
+        <v>0.179666625</v>
       </c>
       <c r="BX6">
-        <v>0.23069465</v>
+        <v>0.22998299999999999</v>
       </c>
       <c r="BY6">
-        <v>0.22642927500000001</v>
+        <v>0.22692085000000001</v>
       </c>
       <c r="BZ6">
-        <v>0.19534499999999999</v>
+        <v>0.19635972500000001</v>
       </c>
       <c r="CA6">
-        <v>0.15549499999999999</v>
+        <v>0.157142</v>
       </c>
       <c r="CB6">
-        <v>0.12049</v>
+        <v>0.12180199999999999</v>
       </c>
       <c r="CC6">
-        <v>5.5584404999999996E-2</v>
+        <v>5.6355299999999997E-2</v>
       </c>
       <c r="CD6">
-        <v>0.14955679999999999</v>
+        <v>0.14839102500000001</v>
       </c>
       <c r="CE6">
-        <v>0.25512800000000002</v>
+        <v>0.25213999999999998</v>
       </c>
       <c r="CF6">
-        <v>0.34090742499999999</v>
+        <v>0.339349075</v>
       </c>
       <c r="CG6">
-        <v>0.36957800000000002</v>
+        <v>0.36865900000000001</v>
       </c>
       <c r="CH6">
-        <v>0.31752812499999999</v>
+        <v>0.31576799999999999</v>
       </c>
       <c r="CI6">
-        <v>0.25135459999999998</v>
+        <v>0.25034195000000004</v>
       </c>
       <c r="CJ6">
-        <v>0.19745199999999999</v>
+        <v>0.196718475</v>
       </c>
       <c r="CK6">
-        <v>0.14694954999999998</v>
+        <v>0.1450534</v>
       </c>
       <c r="CL6">
-        <v>2.8565400000000001E-2</v>
+        <v>2.8819822500000002E-2</v>
       </c>
       <c r="CM6">
-        <v>4.1681212499999995E-2</v>
+        <v>4.1899100000000002E-2</v>
       </c>
       <c r="CN6">
-        <v>7.1177900000000002E-2</v>
+        <v>7.0470000000000005E-2</v>
       </c>
       <c r="CO6">
-        <v>0.12928362500000001</v>
+        <v>0.12959999999999999</v>
       </c>
       <c r="CP6">
-        <v>0.19630062500000001</v>
+        <v>0.197403</v>
       </c>
       <c r="CQ6">
-        <v>0.23727725</v>
+        <v>0.236738</v>
       </c>
       <c r="CR6">
-        <v>0.22667899999999999</v>
+        <v>0.227117025</v>
       </c>
       <c r="CS6">
-        <v>0.19361999999999999</v>
+        <v>0.19425899999999999</v>
       </c>
       <c r="CT6">
-        <v>0.15309542500000001</v>
+        <v>0.15392972500000002</v>
       </c>
       <c r="CU6">
-        <v>5.0908299999999997E-2</v>
+        <v>5.1518805000000001E-2</v>
       </c>
       <c r="CV6">
-        <v>0.122187</v>
+        <v>0.121577875</v>
       </c>
       <c r="CW6">
-        <v>0.19396099999999999</v>
+        <v>0.19107199999999999</v>
       </c>
       <c r="CX6">
-        <v>0.28523500000000002</v>
+        <v>0.28154600000000002</v>
       </c>
       <c r="CY6">
-        <v>0.36154700000000001</v>
+        <v>0.35949205000000001</v>
       </c>
       <c r="CZ6">
-        <v>0.38336085000000003</v>
+        <v>0.38273652499999999</v>
       </c>
       <c r="DA6">
-        <v>0.32802599999999998</v>
+        <v>0.32598500000000002</v>
       </c>
       <c r="DB6">
-        <v>0.25951004999999999</v>
+        <v>0.25811269999999997</v>
       </c>
       <c r="DC6">
-        <v>0.20303465000000001</v>
+        <v>0.20161389999999998</v>
       </c>
     </row>
     <row r="7" spans="1:107" x14ac:dyDescent="0.25">
@@ -11646,322 +11646,322 @@
         <v>16</v>
       </c>
       <c r="B7">
-        <v>1.4722000000000001E-2</v>
+        <v>1.51694E-2</v>
       </c>
       <c r="C7">
-        <v>0.10310900000000001</v>
+        <v>0.10301687499999999</v>
       </c>
       <c r="D7">
-        <v>0.1767002</v>
+        <v>0.174895675</v>
       </c>
       <c r="E7">
-        <v>0.19509299999999999</v>
+        <v>0.19891765</v>
       </c>
       <c r="F7">
-        <v>0.18535799999999999</v>
+        <v>0.19717699999999999</v>
       </c>
       <c r="G7">
-        <v>0.166019</v>
+        <v>0.17688000000000001</v>
       </c>
       <c r="H7">
-        <v>0.13661699999999999</v>
+        <v>0.146062</v>
       </c>
       <c r="I7">
-        <v>9.9699700000000002E-2</v>
+        <v>0.10780195000000001</v>
       </c>
       <c r="J7">
-        <v>8.3956544999999994E-2</v>
+        <v>8.7062700000000007E-2</v>
       </c>
       <c r="K7">
-        <v>0.26926299999999997</v>
+        <v>0.27045119999999995</v>
       </c>
       <c r="L7">
-        <v>0.269549125</v>
+        <v>0.26906600000000003</v>
       </c>
       <c r="M7">
-        <v>0.21271999999999999</v>
+        <v>0.21407499999999999</v>
       </c>
       <c r="N7">
-        <v>0.17702799999999999</v>
+        <v>0.17733099999999999</v>
       </c>
       <c r="O7">
-        <v>0.14329900000000001</v>
+        <v>0.14126900000000001</v>
       </c>
       <c r="P7">
-        <v>0.10422099999999999</v>
+        <v>0.100798</v>
       </c>
       <c r="Q7">
-        <v>6.6681417500000006E-2</v>
+        <v>6.3301545000000001E-2</v>
       </c>
       <c r="R7">
-        <v>1.19481E-2</v>
+        <v>1.22183E-2</v>
       </c>
       <c r="S7">
-        <v>9.4885394999999997E-2</v>
+        <v>9.5473100000000005E-2</v>
       </c>
       <c r="T7">
-        <v>0.18908</v>
+        <v>0.18679000000000001</v>
       </c>
       <c r="U7">
-        <v>0.21555099999999999</v>
+        <v>0.21676300000000001</v>
       </c>
       <c r="V7">
-        <v>0.202325</v>
+        <v>0.20815500000000001</v>
       </c>
       <c r="W7">
-        <v>0.17535355</v>
+        <v>0.18326899999999999</v>
       </c>
       <c r="X7">
-        <v>0.14485700000000001</v>
+        <v>0.15292</v>
       </c>
       <c r="Y7">
-        <v>0.110385175</v>
+        <v>0.117356</v>
       </c>
       <c r="Z7">
-        <v>7.4379569999999992E-2</v>
+        <v>7.9670000000000005E-2</v>
       </c>
       <c r="AA7">
-        <v>7.4274199999999999E-2</v>
+        <v>7.6478277499999997E-2</v>
       </c>
       <c r="AB7">
-        <v>0.26831929999999998</v>
+        <v>0.26949099999999998</v>
       </c>
       <c r="AC7">
-        <v>0.32242599999999999</v>
+        <v>0.32151877500000003</v>
       </c>
       <c r="AD7">
-        <v>0.26496399999999998</v>
+        <v>0.26613300000000001</v>
       </c>
       <c r="AE7">
-        <v>0.215223</v>
+        <v>0.215804</v>
       </c>
       <c r="AF7">
-        <v>0.17738699999999999</v>
+        <v>0.17636199999999999</v>
       </c>
       <c r="AG7">
-        <v>0.13633300000000001</v>
+        <v>0.133688</v>
       </c>
       <c r="AH7">
-        <v>9.3427800000000005E-2</v>
+        <v>9.04581E-2</v>
       </c>
       <c r="AI7">
-        <v>5.6100700000000003E-2</v>
+        <v>5.3304499999999998E-2</v>
       </c>
       <c r="AJ7">
-        <v>1.1229922499999998E-2</v>
+        <v>1.11568E-2</v>
       </c>
       <c r="AK7">
-        <v>7.9491580000000006E-2</v>
+        <v>7.9367737499999994E-2</v>
       </c>
       <c r="AL7">
-        <v>0.18055299999999999</v>
+        <v>0.17851700000000001</v>
       </c>
       <c r="AM7">
-        <v>0.22525115000000001</v>
+        <v>0.22494400000000001</v>
       </c>
       <c r="AN7">
-        <v>0.21487772500000002</v>
+        <v>0.21709442499999998</v>
       </c>
       <c r="AO7">
-        <v>0.18277199999999999</v>
+        <v>0.18736900000000001</v>
       </c>
       <c r="AP7">
-        <v>0.1498467</v>
+        <v>0.15385499999999999</v>
       </c>
       <c r="AQ7">
-        <v>0.11713507499999999</v>
+        <v>0.120451</v>
       </c>
       <c r="AR7">
-        <v>8.3283399999999994E-2</v>
+        <v>8.5836200000000001E-2</v>
       </c>
       <c r="AS7">
-        <v>6.4173599999999997E-2</v>
+        <v>6.5937099999999998E-2</v>
       </c>
       <c r="AT7">
-        <v>0.24417800000000001</v>
+        <v>0.24387600000000001</v>
       </c>
       <c r="AU7">
-        <v>0.34044477499999998</v>
+        <v>0.34207100000000001</v>
       </c>
       <c r="AV7">
-        <v>0.31308852500000001</v>
+        <v>0.31537100000000001</v>
       </c>
       <c r="AW7">
-        <v>0.25280000000000002</v>
+        <v>0.252471</v>
       </c>
       <c r="AX7">
-        <v>0.206124</v>
+        <v>0.20532</v>
       </c>
       <c r="AY7">
-        <v>0.163492</v>
+        <v>0.161298</v>
       </c>
       <c r="AZ7">
-        <v>0.11858399999999999</v>
+        <v>0.11550000000000001</v>
       </c>
       <c r="BA7">
-        <v>7.6319849999999995E-2</v>
+        <v>7.3171700000000006E-2</v>
       </c>
       <c r="BB7">
-        <v>1.5695525000000002E-2</v>
+        <v>1.57272E-2</v>
       </c>
       <c r="BC7">
-        <v>6.1842800000000003E-2</v>
+        <v>6.1540900000000003E-2</v>
       </c>
       <c r="BD7">
-        <v>0.15330079999999999</v>
+        <v>0.152256</v>
       </c>
       <c r="BE7">
-        <v>0.22645612499999998</v>
+        <v>0.22488764999999999</v>
       </c>
       <c r="BF7">
-        <v>0.23352800000000001</v>
+        <v>0.23363767500000002</v>
       </c>
       <c r="BG7">
-        <v>0.205873</v>
+        <v>0.20660957499999999</v>
       </c>
       <c r="BH7">
-        <v>0.166652525</v>
+        <v>0.16816577499999999</v>
       </c>
       <c r="BI7">
-        <v>0.13228352500000001</v>
+        <v>0.13359504999999999</v>
       </c>
       <c r="BJ7">
-        <v>0.10063029999999999</v>
+        <v>0.100601</v>
       </c>
       <c r="BK7">
-        <v>5.9043900000000003E-2</v>
+        <v>5.9846539999999997E-2</v>
       </c>
       <c r="BL7">
-        <v>0.20757999999999999</v>
+        <v>0.20620564999999999</v>
       </c>
       <c r="BM7">
-        <v>0.32280999999999999</v>
+        <v>0.321711425</v>
       </c>
       <c r="BN7">
-        <v>0.36647000000000002</v>
+        <v>0.365373</v>
       </c>
       <c r="BO7">
-        <v>0.31627274999999999</v>
+        <v>0.31577300000000003</v>
       </c>
       <c r="BP7">
-        <v>0.254177025</v>
+        <v>0.25333600000000001</v>
       </c>
       <c r="BQ7">
-        <v>0.20472589999999999</v>
+        <v>0.203513</v>
       </c>
       <c r="BR7">
-        <v>0.15731999999999999</v>
+        <v>0.15388879999999999</v>
       </c>
       <c r="BS7">
-        <v>0.1105442</v>
+        <v>0.10623532499999999</v>
       </c>
       <c r="BT7">
-        <v>2.6464584999999999E-2</v>
+        <v>2.6791599999999999E-2</v>
       </c>
       <c r="BU7">
-        <v>4.9519399999999998E-2</v>
+        <v>4.91379225E-2</v>
       </c>
       <c r="BV7">
-        <v>0.114235</v>
+        <v>0.11307135</v>
       </c>
       <c r="BW7">
-        <v>0.19633400000000001</v>
+        <v>0.19503000000000001</v>
       </c>
       <c r="BX7">
-        <v>0.24734500000000001</v>
+        <v>0.24627732499999999</v>
       </c>
       <c r="BY7">
-        <v>0.24018999999999999</v>
+        <v>0.239956</v>
       </c>
       <c r="BZ7">
-        <v>0.20613567500000002</v>
+        <v>0.206209</v>
       </c>
       <c r="CA7">
-        <v>0.16517537499999999</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="CB7">
-        <v>0.13044900000000001</v>
+        <v>0.1292981</v>
       </c>
       <c r="CC7">
-        <v>6.1710302500000001E-2</v>
+        <v>6.2118699999999999E-2</v>
       </c>
       <c r="CD7">
-        <v>0.165079375</v>
+        <v>0.16341344999999999</v>
       </c>
       <c r="CE7">
-        <v>0.273381975</v>
+        <v>0.27112802499999999</v>
       </c>
       <c r="CF7">
-        <v>0.35994399999999999</v>
+        <v>0.35782999999999998</v>
       </c>
       <c r="CG7">
-        <v>0.39113399999999998</v>
+        <v>0.38833499999999999</v>
       </c>
       <c r="CH7">
-        <v>0.33599000000000001</v>
+        <v>0.333594</v>
       </c>
       <c r="CI7">
-        <v>0.27026499999999998</v>
+        <v>0.26854662500000004</v>
       </c>
       <c r="CJ7">
-        <v>0.215087</v>
+        <v>0.21220702499999999</v>
       </c>
       <c r="CK7">
-        <v>0.16389799999999999</v>
+        <v>0.15914910000000002</v>
       </c>
       <c r="CL7">
-        <v>3.0136234999999997E-2</v>
+        <v>3.02701425E-2</v>
       </c>
       <c r="CM7">
-        <v>4.5541600000000002E-2</v>
+        <v>4.5363399999999998E-2</v>
       </c>
       <c r="CN7">
-        <v>8.0206594999999992E-2</v>
+        <v>7.9187044999999998E-2</v>
       </c>
       <c r="CO7">
-        <v>0.14427252500000001</v>
+        <v>0.14344100000000001</v>
       </c>
       <c r="CP7">
-        <v>0.21369199999999999</v>
+        <v>0.21295</v>
       </c>
       <c r="CQ7">
-        <v>0.25215199999999999</v>
+        <v>0.25134699999999999</v>
       </c>
       <c r="CR7">
-        <v>0.23924699999999999</v>
+        <v>0.23904700000000001</v>
       </c>
       <c r="CS7">
-        <v>0.203582175</v>
+        <v>0.20297000000000001</v>
       </c>
       <c r="CT7">
-        <v>0.16214527500000001</v>
+        <v>0.160795825</v>
       </c>
       <c r="CU7">
-        <v>5.5677299999999999E-2</v>
+        <v>5.6346599999999997E-2</v>
       </c>
       <c r="CV7">
-        <v>0.13607897499999999</v>
+        <v>0.135812025</v>
       </c>
       <c r="CW7">
-        <v>0.21307699999999999</v>
+        <v>0.2106191</v>
       </c>
       <c r="CX7">
-        <v>0.304412075</v>
+        <v>0.30171337500000001</v>
       </c>
       <c r="CY7">
-        <v>0.3821</v>
+        <v>0.37889099999999998</v>
       </c>
       <c r="CZ7">
-        <v>0.40545437499999998</v>
+        <v>0.40191690000000002</v>
       </c>
       <c r="DA7">
-        <v>0.34779300000000002</v>
+        <v>0.34425905000000001</v>
       </c>
       <c r="DB7">
-        <v>0.278207025</v>
+        <v>0.27598455</v>
       </c>
       <c r="DC7">
-        <v>0.22150400000000001</v>
+        <v>0.21746499999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>